<commit_message>
Updates from testing ABS vehicle.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@21904 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/SGMW/SGMW Plant Matrix.xlsx
+++ b/Source/SGMW/SGMW Plant Matrix.xlsx
@@ -460,7 +460,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -570,6 +570,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -1058,10 +1061,10 @@
         <v>34</v>
       </c>
       <c r="F19" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="45" t="s">
         <v>31</v>
-      </c>
-      <c r="G19" s="43" t="s">
-        <v>36</v>
       </c>
       <c r="H19" s="43" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Updates from debugging software and test cycles.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@21952 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/SGMW/SGMW Plant Matrix.xlsx
+++ b/Source/SGMW/SGMW Plant Matrix.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="46">
   <si>
     <t>S / N</t>
   </si>
@@ -148,6 +148,12 @@
   </si>
   <si>
     <t>172.16.250.2</t>
+  </si>
+  <si>
+    <t>508497-01</t>
+  </si>
+  <si>
+    <t>10.18.13.27</t>
   </si>
 </sst>
 </file>
@@ -993,6 +999,9 @@
     </row>
     <row r="17" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
+      <c r="H17" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="18" spans="1:17" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
@@ -1092,21 +1101,47 @@
       <c r="Q19" s="24"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="G20" s="43"/>
-      <c r="H20" t="s">
-        <v>42</v>
+      <c r="A20" s="14">
+        <v>2</v>
+      </c>
+      <c r="B20" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="5">
+        <v>3700</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="I20" s="45" t="s">
+        <v>43</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
+      <c r="L20" s="43" t="s">
+        <v>37</v>
+      </c>
+      <c r="M20" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="N20" s="5">
+        <v>50849701</v>
+      </c>
+      <c r="O20" s="43" t="s">
+        <v>39</v>
+      </c>
       <c r="P20" s="18"/>
       <c r="Q20" s="24"/>
     </row>

</xml_diff>